<commit_message>
fix(security): 의존성 취약점과 공개 레포 개인 경로 제거 (v0.8.23, SYM-97 SYM-98)
requirements.txt 가 하한만 두어 pypdf 6.9.2, requests 2.32.5 가 설치돼
있었다. pypdf 는 조작된 PDF 로 장시간 실행이나 메모리 고갈을 유발하는
취약점 47건에 해당한다. Slack 첨부를 그대로 파싱하므로 채널 참여자가
봇을 멈출 수 있었다. 하한을 pypdf>=6.18.1, requests>=2.34.2 로 올린다.

공개 레포 추적 파일 9곳에 남아 있던 로컬 절대경로를 제거한다. Windows
사용자명과 홈 구조, 보유 프로젝트명이 드러나던 자리다. 문서와 테스트는
플레이스홀더로 바꾸고, 기동 스크립트 둘은 자기 위치 기준으로 고친다.
start_watchdog.vbs 주석은 ASCII 로 둔다. WSH 가 UTF-8 을 읽지 못한다.

OSV: pypdf 47건 -> 0건, requests 2건 -> 0건
검증: pytest 487건 통과, ps1 파싱 확인
issue_log.xlsx 는 OPENPYXL_LXML=False 로 저장하고 전 셀 2,537개를 대조했다

git 히스토리에는 경로가 남으므로 효과는 앞으로의 노출 축소에 한정된다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -421,8 +421,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V150"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:V152"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -9208,7 +9208,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>1. 토론 채널에서 'C:\Users\ymseo\Documents\sym-ui 경로의 프로젝트를 평가해줘' 류 주제 투입 2. Codex(codex exec -s workspace-write)가 cwd 밖 경로 접근 시도 → Windows exited -1073741502(0xC0000142 STATUS_DLL_INIT_FAILED)로 자식 프로세스 시작 실패 3. Gemini/Claude 는 정상 분석, Codex 만 '권한 문제'처럼 보이며 평가 보류</t>
+          <t>1. 토론 채널에서 'C:\work\sym-ui 경로의 프로젝트를 평가해줘' 류 주제 투입 2. Codex(codex exec -s workspace-write)가 cwd 밖 경로 접근 시도 → Windows exited -1073741502(0xC0000142 STATUS_DLL_INIT_FAILED)로 자식 프로세스 시작 실패 3. Gemini/Claude 는 정상 분석, Codex 만 '권한 문제'처럼 보이며 평가 보류</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -11278,6 +11278,227 @@
       </c>
       <c r="U150" t="n">
         <v>147</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>requirements 하한이 낮아 pypdf 가 조작된 PDF 에 DoS 되는 버전으로 설치된다</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>- requirements.txt 가 pypdf&gt;=4.0, requests&gt;=2.31.0 처럼 하한만 두어 취약 버전이 설치돼 있었다.
+- pypdf 6.9.2 에 조작된 PDF 로 장시간 실행이나 메모리 고갈을 유발하는 취약점 47건이 있다.
+- requests 2.32.5 는 extract_zipped_paths 의 임시파일 재사용(GHSA-gc5v-m9x4-r6x2) 등 2건.</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>- Slack 으로 들어온 첨부를 파싱하는 의존성에 알려진 취약점이 없어야 한다.</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>- OSV 조회 결과 pypdf 47건, requests 2건.</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>- 봇이 Slack 첨부 PDF 를 pypdf 로 파싱하므로, 채널에 올린 파일이 그대로 파서 입력이 된다.</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>1. requirements.txt 에서 pypdf 와 requests 가 하한만 지정된 것을 확인
+2. pip show 로 설치 버전 확인 (pypdf 6.9.2, requests 2.32.5)
+3. OSV API 에 각 패키지와 버전으로 조회</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>- OSV API 응답. pypdf 취약점 다수가 6.10.x~6.16.x 구간에서 순차 수정됨.</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. 전체 프로젝트 보안 점검 중 확인.</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>원인: - requirements.txt 를 하한(&gt;=)으로만 관리해 취약 버전이 그대로 남았다.
+수정 내용: - requests&gt;=2.34.2, pypdf&gt;=6.18.1 로 하한을 올리고 사유를 주석으로 남겼다.
+- 설치 후 OSV 재조회 둘 다 0건
+- pytest 487건 통과</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>- 하한 상향이 가드다. 다만 하한 방식은 시간이 지나면 다시 벌어지므로 주기 점검이 필요하다.</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>- Slack 첨부 PDF 파싱 경로. 채널 참여자가 조작된 PDF 로 봇을 멈출 수 있었다.</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>v0.8.22</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>- v0.8.23</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>SYM-97</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>공개 레포에 로컬 절대경로가 남아 Windows 사용자명과 홈 구조가 노출된다</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>- public 레포 sym804/ai-squad 의 추적 파일 9곳에 C:\Users\&lt;user&gt;\... 가 남아 있다.
+- Windows 사용자명, 홈 디렉터리 구조, 보유 프로젝트명(stockradar, sym-ui), .gemini 확장 설치 내역이 드러난다.
+- 대상: RELEASE_NOTES.md, agents/codex.py 주석, docs/2026-04-02-implementation-plan.md, tests/test_security.py, tests/test_debate_cwd.py, tests/test_codex_last_message.py, tests/test_gemini.py, migrate_session0.ps1, start_watchdog.vbs, issue_log.xlsx.</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>- 공개 레포 추적 파일에 개인 절대경로가 없어야 한다.</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>- 단일 백슬래시 형태 15곳, 소스에 이스케이프된 이중 백슬래시 형태 4곳, xlsx 내부 1곳.</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>1. git ls-files 로 추적 파일 목록을 뽑는다
+2. 각 파일에서 C:\Users\&lt;user&gt; 를 단일/이중 백슬래시 두 형태로 찾는다
+3. xlsx 는 zip 이므로 압축을 풀어 sheet xml 까지 본다</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>- 추적 파일 74개 전수 스캔 결과. issue_log.xlsx 는 xl/worksheets/sheet1.xml 의 K122 셀.</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. 전체 프로젝트 보안 점검 중 확인.</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>원인: - 로컬에서 쓰던 경로를 그대로 커밋했다. 같은 유형이 claude-config 에서 한 번 정리된 적 있는데 이 레포는 남아 있었다.
+수정 내용: - 문서와 테스트의 경로를 C:\work\... 또는 플레이스홀더로 치환했다.
+- migrate_session0.ps1 은 폴백을 Get-Location 으로, 실행 예시에 cd 전제를 명시했다.
+- start_watchdog.vbs 는 자기 위치 기준(WScript.ScriptFullName)으로 바꿨다. WSH 가 UTF-8 을 못 읽으므로 주석은 ASCII 로 유지했다.
+- issue_log.xlsx 는 OPENPYXL_LXML=False 로 저장하고 전 셀 2,537개를 대조해 무손실 확인했다.
+- pytest 487건 통과.</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>- 붙이지 않았다. pre-commit 에 xlsx 언집을 포함한 개인정보 스캔 훅을 거는 것이 근본 처방이나 별도 작업이다.</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>- git 히스토리에는 그대로 남으므로 이 수정의 효과는 앞으로의 노출 축소에 한정된다.</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>v0.8.22</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>- v0.8.23</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>SYM-98</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>